<commit_message>
Fix IŞIK PETROL ZİRAAT commission calculation (6069 rows)
- 01.06.2026 - 10.06.2026: 1296 işlem, 34819.02 TL
- 11.06.2026 - 20.06.2026: 2826 işlem, 73137.49 TL
- 21.06.2026 - 30.06.2026: 1883 işlem, 113858.33 TL
- Genel Toplam: 6005 işlem, 221814.84 TL

Fixed regex pattern to correctly extract commission values from descriptions
</commit_message>
<xml_diff>
--- a/ISIK_PETROL_ZIRAAT_KOMISYON_OZET.xlsx
+++ b/ISIK_PETROL_ZIRAAT_KOMISYON_OZET.xlsx
@@ -488,10 +488,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>84</v>
+        <v>1296</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>695.39</v>
+        <v>34819.01999999997</v>
       </c>
     </row>
     <row r="3">
@@ -501,10 +501,10 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>182</v>
+        <v>2826</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>3430.359999999998</v>
+        <v>73137.48999999986</v>
       </c>
     </row>
     <row r="4">
@@ -514,10 +514,10 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>154</v>
+        <v>1883</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>3185.63</v>
+        <v>113858.33</v>
       </c>
     </row>
     <row r="6">
@@ -527,10 +527,10 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>420</v>
+        <v>6005</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>7311.379999999998</v>
+        <v>221814.8399999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>